<commit_message>
Fix patient and location QR lookup
</commit_message>
<xml_diff>
--- a/outputs/russicaptor-mimino-12/Mimino_Botulism_12_Patients.xlsx
+++ b/outputs/russicaptor-mimino-12/Mimino_Botulism_12_Patients.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R5867a30dfc134f4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patients" sheetId="2" r:id="R579da1efe0f94556"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Locations" sheetId="3" r:id="R008b918907d54894"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="InterventionOptions" sheetId="4" r:id="R07032625273f474c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interventions" sheetId="5" r:id="Rc595355d116b47fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MedicationOptions" sheetId="6" r:id="Rada7aa0b56c54a05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MedicationAdministrations" sheetId="7" r:id="Rd3a0d1d2f70c48fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vitals" sheetId="8" r:id="R06cdb8dd6d654a95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="9" r:id="Rdf813e30141741d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Labs" sheetId="10" r:id="R72bb6502061f4f97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Imaging" sheetId="11" r:id="Ree2188b568324370"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="12" r:id="Rc089b19ed92e48c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orders" sheetId="13" r:id="R123c679f01c64c37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="Rd7fc837e97de4fb2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patients" sheetId="2" r:id="R9a37822f96cf463c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Locations" sheetId="3" r:id="Rf379202fd9d54556"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="InterventionOptions" sheetId="4" r:id="R6ca42edf212d4bf7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interventions" sheetId="5" r:id="Rb426ea65499149a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MedicationOptions" sheetId="6" r:id="R73126127c95d4638"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MedicationAdministrations" sheetId="7" r:id="R8524ef821a414d1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vitals" sheetId="8" r:id="R8ff8bcd2a21b459b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="9" r:id="R745e274c972744e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Labs" sheetId="10" r:id="Rbeb9f29c92cb4110"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Imaging" sheetId="11" r:id="R995cf4f5e3de4526"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="12" r:id="Rc07fb9204aa04337"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orders" sheetId="13" r:id="R51ad1dadc4bd486c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25,6 +25,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="@"/>
+  </x:numFmts>
   <x:fonts count="5">
     <x:font>
       <x:sz val="11"/>
@@ -131,7 +134,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="26">
+  <x:cellXfs count="27">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -180,6 +183,9 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -190,7 +196,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5E9"/>
         </x:patternFill>
       </x:fill>
@@ -578,7 +584,7 @@
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
       <x:c r="A3" s="21" t="str">
-        <x:v>Fiktiivsed õppuse patsiendid. Andmed on täiendatud MIMINO stsenaariumi meditsiinilise loogika järgi. Kõik SIM-MIMINO-* tunnused on sünteetilised QR-väärtused.</x:v>
+        <x:v>Fiktiivsed õppuse patsiendid. Andmed on täiendatud MIMINO stsenaariumi meditsiinilise loogika järgi. NationalId väärtused on genereeritud Eesti isikukoodi struktuuri ja kontrollnumbri reeglite järgi.</x:v>
       </x:c>
       <x:c r="B3" s="21"/>
       <x:c r="C3" s="21"/>
@@ -2050,7 +2056,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2ed2b15429a4b4c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69ec7c818a5a4ffa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2196,7 +2202,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf76bd2221dd34bda"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd2b3818b6464b70"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2875,7 +2881,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb04fffe0e7d44a44"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49bf7ddeed5a4664"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2943,8 +2949,8 @@
       <x:c r="B2" s="16" t="str">
         <x:v>P01</x:v>
       </x:c>
-      <x:c r="C2" s="16" t="str">
-        <x:v>SIM-MIMINO-P01</x:v>
+      <x:c r="C2" s="26" t="str">
+        <x:v>37203140017</x:v>
       </x:c>
       <x:c r="D2" s="16" t="str">
         <x:v>Tarmo Lepp</x:v>
@@ -2981,8 +2987,8 @@
       <x:c r="B3" s="16" t="str">
         <x:v>P02</x:v>
       </x:c>
-      <x:c r="C3" s="16" t="str">
-        <x:v>SIM-MIMINO-P02</x:v>
+      <x:c r="C3" s="26" t="str">
+        <x:v>45411020027</x:v>
       </x:c>
       <x:c r="D3" s="16" t="str">
         <x:v>Leida Saar</x:v>
@@ -3019,8 +3025,8 @@
       <x:c r="B4" s="16" t="str">
         <x:v>P03</x:v>
       </x:c>
-      <x:c r="C4" s="16" t="str">
-        <x:v>SIM-MIMINO-P03</x:v>
+      <x:c r="C4" s="26" t="str">
+        <x:v>37706210032</x:v>
       </x:c>
       <x:c r="D4" s="16" t="str">
         <x:v>Andres Kask</x:v>
@@ -3057,8 +3063,8 @@
       <x:c r="B5" s="16" t="str">
         <x:v>P04</x:v>
       </x:c>
-      <x:c r="C5" s="16" t="str">
-        <x:v>SIM-MIMINO-P04</x:v>
+      <x:c r="C5" s="26" t="str">
+        <x:v>48004080041</x:v>
       </x:c>
       <x:c r="D5" s="16" t="str">
         <x:v>Kadri Kask</x:v>
@@ -3095,8 +3101,8 @@
       <x:c r="B6" s="16" t="str">
         <x:v>P05</x:v>
       </x:c>
-      <x:c r="C6" s="16" t="str">
-        <x:v>SIM-MIMINO-P05</x:v>
+      <x:c r="C6" s="26" t="str">
+        <x:v>60809170053</x:v>
       </x:c>
       <x:c r="D6" s="16" t="str">
         <x:v>Liisa Kask</x:v>
@@ -3133,8 +3139,8 @@
       <x:c r="B7" s="16" t="str">
         <x:v>P06</x:v>
       </x:c>
-      <x:c r="C7" s="16" t="str">
-        <x:v>SIM-MIMINO-P06</x:v>
+      <x:c r="C7" s="26" t="str">
+        <x:v>51401250060</x:v>
       </x:c>
       <x:c r="D7" s="16" t="str">
         <x:v>Martin Kask</x:v>
@@ -3171,8 +3177,8 @@
       <x:c r="B8" s="16" t="str">
         <x:v>P07</x:v>
       </x:c>
-      <x:c r="C8" s="16" t="str">
-        <x:v>SIM-MIMINO-P07</x:v>
+      <x:c r="C8" s="26" t="str">
+        <x:v>38408300078</x:v>
       </x:c>
       <x:c r="D8" s="16" t="str">
         <x:v>Toomas Vaher</x:v>
@@ -3209,8 +3215,8 @@
       <x:c r="B9" s="16" t="str">
         <x:v>P08</x:v>
       </x:c>
-      <x:c r="C9" s="16" t="str">
-        <x:v>SIM-MIMINO-P08</x:v>
+      <x:c r="C9" s="26" t="str">
+        <x:v>48612120083</x:v>
       </x:c>
       <x:c r="D9" s="16" t="str">
         <x:v>Anneli Põld</x:v>
@@ -3247,8 +3253,8 @@
       <x:c r="B10" s="16" t="str">
         <x:v>P09</x:v>
       </x:c>
-      <x:c r="C10" s="16" t="str">
-        <x:v>SIM-MIMINO-P09</x:v>
+      <x:c r="C10" s="26" t="str">
+        <x:v>38205190097</x:v>
       </x:c>
       <x:c r="D10" s="16" t="str">
         <x:v>Raivo Mets</x:v>
@@ -3285,8 +3291,8 @@
       <x:c r="B11" s="16" t="str">
         <x:v>P10</x:v>
       </x:c>
-      <x:c r="C11" s="16" t="str">
-        <x:v>SIM-MIMINO-P10</x:v>
+      <x:c r="C11" s="26" t="str">
+        <x:v>49807040108</x:v>
       </x:c>
       <x:c r="D11" s="16" t="str">
         <x:v>Laura Tamm</x:v>
@@ -3323,8 +3329,8 @@
       <x:c r="B12" s="16" t="str">
         <x:v>P11</x:v>
       </x:c>
-      <x:c r="C12" s="16" t="str">
-        <x:v>SIM-MIMINO-P11</x:v>
+      <x:c r="C12" s="26" t="str">
+        <x:v>39410230113</x:v>
       </x:c>
       <x:c r="D12" s="16" t="str">
         <x:v>Markus Tamm</x:v>
@@ -3361,8 +3367,8 @@
       <x:c r="B13" s="16" t="str">
         <x:v>P12</x:v>
       </x:c>
-      <x:c r="C13" s="16" t="str">
-        <x:v>SIM-MIMINO-P12</x:v>
+      <x:c r="C13" s="26" t="str">
+        <x:v>35202160120</x:v>
       </x:c>
       <x:c r="D13" s="16" t="str">
         <x:v>Heino Oja</x:v>
@@ -3395,7 +3401,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb230c1998f1947fa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41282da57bd049ac"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3531,7 +3537,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f78365983d54b6a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1abab9ae73d042a4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3971,7 +3977,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Read3be545ebf449c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa90925c53b442ff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4520,7 +4526,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71c87a43c0864f2d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a3cdc7621d24917"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5901,7 +5907,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9def93cef458427f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3130328213f641f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7197,7 +7203,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raebc490d88d14158"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5143d63279d34d30"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>